<commit_message>
daily rejection graph updated
</commit_message>
<xml_diff>
--- a/rods.xlsx
+++ b/rods.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X81"/>
+  <dimension ref="A1:X82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5601,10 +5601,8 @@
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M81" t="n">
+        <v>1</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
@@ -5659,6 +5657,78 @@
       <c r="X81" t="inlineStr">
         <is>
           <t>cvcv</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="n">
+        <v>1</v>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>sd</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>suyashh</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>zx</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>zv</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>zcxvb</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>zxvb</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>vbx c</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>xvb</t>
+        </is>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>zfv</t>
         </is>
       </c>
     </row>

</xml_diff>